<commit_message>
updated all files to include context file in the prompts
</commit_message>
<xml_diff>
--- a/docs/User story.xlsx
+++ b/docs/User story.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -27,16 +27,39 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
+    <font/>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F7FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -44,11 +67,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -56,6 +94,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,7 +511,7 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="51.7109375" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
     <col width="80" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
@@ -465,56 +519,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>User story</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>BDD test cases</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="8" t="inlineStr">
         <is>
           <t>Classic test cases</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="409.5" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Title: [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout
 As a Product Owner, I want to start a Black Friday campaign, so that we increase our revenue on the "Smartphone-Shop" website.
-The Black Friday campaign has a "BF2026" coupon code - 20% discount already applied at checkout.
+The Black Friday campaign has a "BF2026" coupon code - 20% discount only per one unit of product.
+Products can be Android and iOS smarphones and their specific accesories (casses, screen protectors, cables and charges).
 The period of the promotion is between 2026-11-27 00:00 to 2026-11-30 23:59:59 (shop local time, Europe/Bucharest).
-The coupon code can be applied only once for 1 Quantity of that product on one user_ID.
+The coupon code can be applied only once per 1 unit of the same product per user_ID.
 Example: you can purchase only 1 Samsung Galaxy S26 Ultra 512GB Smartphone with coupon code: "BF2026" on user_ID=5456.
 Data Mapping:
 Promotion name: BlackFriday2026
-Coupon code : "BF2026" is a 20% discount from the total amount at checkout
+Coupon code : "BF2026" is a 20% discount per 1 unit
 Period: between 2026-11-27 00:00 to 2026-11-30 23:59:59 (shop local time, Europe/Bucharest).
 Users: any registered users on the Smartphone-Shop
 Usage Limit per Customer: Coupon code is applied per 1 QTY of the same product for only 1 user_ID.
 Validation: On Checkout "BF2026" is not case sensitive, all other coupon codes are not available.
 AC1: Discount is applied
-GIVEN that I'm a User
+GIVEN that I'm a registered User
 WHEN I am at the Checkout page
-AND I purchase 1QTY of product
+AND I purchase 1 unit of the product (smarphone, case, cable, charger)
 I apply coupon code "BF2026"
-THEN The 20% discount is applied for the total amount.
+THEN The 20% discount is applied per 1 unit.
 AC2: Discount is not applied for two units of same products
-GIVEN that I'm a User
+GIVEN that I'm a registered User
 WHEN I am at the Checkout page
 AND I purchase 2 units of the same product with coupon code "BF2026"
 THEN The 20% discount is applied only on 1 unit
@@ -523,17 +578,13 @@
 GIVEN that I'm an User at the Checkout page
 WHEN I enter any coupon code other than “BF2026” (e.g., “BF2025”, “SAVE10”),
 THEN the system displays “This coupon is not valid” and no discount is applied.
-AC4: Guest users cannot use the coupon
-GIVEN I'm a Guest
-WHEN they try to apply “BF2026”,
-THEN the system displays “Please log in to use this coupon” and no discount is applied.
-AC5: Successful order
+AC4: Successful order
 GIVEN that I'm a User that completes the payment with “BF2026” applied,
 WHEN the order is confirmed,
 THEN the system stores a redemption record, with coupon code “BF2026”, user_ID, product_ID, quantity discounted = 1, discount amount, and a UTC timestamp.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>- Q1: Which products are eligible: all smartphones and accessories in the catalog, or only specific categories? Are screen protectors included (they are in the description but not in AC1)? — Expected: the list of categories, and the exclusions (out-of-stock, pre-order, already discounted).
 - Q2: What identifies "the same product": product_ID, or product_ID plus variant (color, storage)? Is a Samsung Galaxy S26 Ultra 512GB the same product as the 256GB version? — Expected: the rule based on product_ID or SKU.
@@ -544,18 +595,17 @@
 - Q7: Which timezone and boundary rules apply (Europe/Bucharest is UTC+2 in November)? Is 2026-11-30 23:59:59 inclusive, and which clock is used (server)? — Expected: inclusive boundaries, server time.
 - Q8: Is the code case-insensitive only for letters, or is it also trimmed for spaces? Are "bf2026", " BF2026 ", and "BF-2026" valid? — Expected: the accepted-input rules.
 - Q9: Is the "This coupon is not valid" message the same for an empty code, an expired code, and an unknown code? Is there a limit on invalid attempts? — Expected: messages and rate limiting.
-- Q10: What happens to a guest after "Please log in to use this coupon"? Is the cart preserved and the coupon re-applied after login or registration? — Expected: the flow after login.
-- Q11: If payment fails or the user abandons checkout, is the coupon reserved or released? What about order cancellation, refund, or partial return of the discounted unit? Is the redemption record deleted, flagged, or kept? — Expected: the rule for each case.
-- Q12: What happens with two simultaneous checkouts (two tabs, two devices) of the same user for the same product? — Expected: only one succeeds.
-- Q13: Does the coupon combine with existing product discounts, sale prices, or other vouchers? — Expected: stackable or not.
-- Q14: How is the 20% calculated (before or after VAT and shipping), and what is the rounding rule and currency? — Expected: formula and rounding (e.g., 2 decimals, half-up).
-- Q15: Which UI elements show the discount (line item, new total, applied coupon label), and can the user remove the coupon? — Expected: UI/UX specification or mockup.
-- Q16: What exactly is stored in the redemption record (discount amount with or without VAT, currency, order_ID), and how can testers check it (DB, API, report)? — Expected: schema and an access method.
-- Q17: Is there a way to change the system date and to prepare test data (registered users, products, stock) in the test environment? — Expected: environment and mocking support, or a feature flag.
-- Q18: Are NFRs in scope (load on Black Friday, security of the coupon endpoint, accessibility, localization of messages, supported browsers and mobile)? — Expected: in or out of scope.</t>
+- Q10: If payment fails or the user abandons checkout, is the coupon reserved or released? What about order cancellation, refund, or partial return of the discounted unit? Is the redemption record deleted, flagged, or kept? — Expected: the rule for each case.
+- Q11: What happens with two simultaneous checkouts (two tabs, two devices) of the same user for the same product? — Expected: only one succeeds.
+- Q12: Does the coupon combine with existing product discounts, sale prices, or other vouchers? — Expected: stackable or not.
+- Q13: How is the 20% calculated (before or after VAT and shipping), and what is the rounding rule and currency? — Expected: formula and rounding (e.g., 2 decimals, half-up).
+- Q14: Which UI elements show the discount (line item, new total, applied coupon label), and can the user remove the coupon? — Expected: UI/UX specification or mockup.
+- Q15: What exactly is stored in the redemption record (discount amount with or without VAT, currency, order_ID), and how can testers check it (DB, API, report)? — Expected: schema and an access method.
+- Q16: Is there a way to change the system date and to prepare test data (registered users, products, stock) in the test environment? — Expected: environment and mocking support, or a feature flag.
+- Q17: Are NFRs in scope (load on Black Friday, security of the coupon endpoint, accessibility, localization of messages, supported browsers and mobile)? — Expected: in or out of scope.</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>#### AC1 – Discount is applied (registered user, 1 unit)
 - [ ] [AC1] Check that a registered user with 1 unit of a smartphone in the cart gets 20% off that unit after applying "BF2026" at Checkout during the promotion period
@@ -592,20 +642,14 @@
 - [ ] [AC3] Check the behavior with special characters, emojis, a very long string, SQL injection, and script injection (no error, no stored XSS, safe message)
 - [ ] [AC3] Check that an invalid code attempt does not remove an already applied valid "BF2026"
 - [ ] [AC3] Check that the message text matches exactly “This coupon is not valid” (and its localization)
-#### AC4 – Guest users
-- [ ] [AC4] Check that a guest applying "BF2026" sees “Please log in to use this coupon” and no discount is applied
-- [ ] [AC4] Check that a guest applying an invalid code sees “This coupon is not valid” (or the login message, per the answer)
-- [ ] [AC4] Check that after login or registration, the cart is preserved and the coupon can be applied
-- [ ] [AC4] Check that a user whose session expired at Checkout is treated as a guest
-- [ ] [AC4] Check that a guest cannot get the discount by calling the coupon API directly
-#### AC5 – Successful order and redemption record
-- [ ] [AC5] Check that after payment and order confirmation, a redemption record is stored with coupon code "BF2026", the correct user_ID, product_ID, quantity discounted = 1, the discount amount, and a UTC timestamp
-- [ ] [AC5] Check that the discount amount in the record equals the discount shown in the order and the invoice
-- [ ] [AC5] Check that the UTC timestamp is correct (Europe/Bucharest local time minus 2 hours in November)
-- [ ] [AC5] Check that with qty 2 only one redemption record (quantity discounted = 1) is stored
-- [ ] [AC5] Check that with a cart of several products, one record per discounted product is stored
-- [ ] [AC5] Check that no redemption record is stored for failed, cancelled, or abandoned orders
-- [ ] [AC5] Check that the order confirmation page, email, and order history show the discounted price
+#### AC4 – Successful order and redemption record
+- [ ] [AC4] Check that after payment and order confirmation, a redemption record is stored with coupon code "BF2026", the correct user_ID, product_ID, quantity discounted = 1, the discount amount, and a UTC timestamp
+- [ ] [AC4] Check that the discount amount in the record equals the discount shown in the order and the invoice
+- [ ] [AC4] Check that the UTC timestamp is correct (Europe/Bucharest local time minus 2 hours in November)
+- [ ] [AC4] Check that with qty 2 only one redemption record (quantity discounted = 1) is stored
+- [ ] [AC4] Check that with a cart of several products, one record per discounted product is stored
+- [ ] [AC4] Check that no redemption record is stored for failed, cancelled, or abandoned orders
+- [ ] [AC4] Check that the order confirmation page, email, and order history show the discounted price
 #### Promotion period
 - [ ] [Period] Check that "BF2026" is accepted at 2026-11-27 00:00:00 and rejected at 2026-11-26 23:59:59 (shop local time)
 - [ ] [Period] Check that "BF2026" is accepted at 2026-11-30 23:59:59 and rejected at 2026-12-01 00:00:00
@@ -631,18 +675,24 @@
 - [ ] [Localization] Check that messages are shown in the correct language and currency format
 #### Environment / Configuration
 - [ ] [Env] Check that the test environment can set the system date inside and outside of the period
-- [ ] [Env] Check that test data exist: registered users, a guest session, Android/iOS products, and each accessory type
+- [ ] [Env] Check that test data exist: registered users, Android/iOS products, and each accessory type
 - [ ] [Env] Check that the redemption records can be viewed (DB, API, or report) in the test environment
 - [ ] [Env] Check that the coupon is not available in the production environment before the start date
 #### Regression
 - [ ] [Regression] Check that checkout without a coupon still calculates totals, VAT, shipping, and rounding correctly
 - [ ] [Regression] Check that existing promotions and discounts still work
-- [ ] [Regression] Check that guest checkout, login, and registration still work
+- [ ] [Regression] Check that login and registration still work
 - [ ] [Regression] Check that order history, invoices, emails, and order cancellation/refund still show correct amounts
-- [ ] [Regression] Check that reports and analytics still work with the new redemption records</t>
+- [ ] [Regression] Check that reports and analytics still work with the new redemption records
+#### Short checklist (5 items)
+- [ ] [AC1/AC2] Check that a logged-in customer (user_ID 5456) with 2 units of "Samsung Galaxy S26 Ultra 512GB" at 1000.00 each gets 20% off only 1 unit after applying "BF2026" (any letter case, such as "bf2026") at Checkout. The discount is 200.00, the second unit stays at 1000.00, the total is 1800.00, and the cart, order summary and Stripe amount all match.
+- [ ] [AC3] Check that "BF2025", "SAVE10", an empty code, and injection strings (`' OR '1'='1`, `&lt;script&gt;`) show "This coupon is not valid" and apply no discount. Also check that a failed attempt does not remove an already applied valid "BF2026".
+- [ ] [Period] Check that the server time (Europe/Bucharest, UTC+2) decides validity: accepted at 2026-11-27 00:00:00 and 2026-11-30 23:59:59, rejected at 2026-11-26 23:59:59 and 2026-12-01 00:00:00, and not affected by the user's device clock.
+- [ ] [AC4/Usage limit] Check that after payment and order confirmation exactly 1 redemption record is stored (coupon code "BF2026", user_ID, product_ID, quantity discounted = 1, discount amount 200.00, UTC timestamp). Also check that a second order by the same user for the same product is rejected, that a failed or cancelled payment stores no record, and that a double-click on "Pay" or a payment webhook retry does not create a duplicate.
+- [ ] [Security] Check that the discount cannot be changed by tampering with the request (price, discount percent, quantity, user_ID). The server must recalculate the price, reject unauthenticated or expired-token coupon requests, and rate limit repeated invalid attempts.</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>Feature: Apply Black Friday coupon code "BF2026" at checkout (STORY-1347)
   Background:
@@ -773,29 +823,8 @@
       | ' OR '1'='1               |
       | &lt;script&gt;alert(1)&lt;/script&gt; |
       | 5000 characters string    |
-  # ---------- AC4: Guest users (3) ----------
-  @High @Negative @RoleBased @AC4
-  Scenario: Guest cannot use the coupon
-    Given I am a guest at the Checkout page with 1 unit of a product
-    When I apply the coupon code "BF2026"
-    Then the message "Please log in to use this coupon" is displayed
-    And no discount is applied
-  @Medium @Alternate @AC4
-  Scenario: Guest logs in and applies the coupon
-    Given I am a guest at the Checkout page with 1 unit of a product
-    And I saw the message "Please log in to use this coupon"
-    When I log in as a registered user
-    And I apply the coupon code "BF2026"
-    Then my cart is preserved
-    And the 20% discount is applied to the unit
-  @High @Security @AC4
-  Scenario: Guest cannot apply the coupon by calling the API directly
-    Given I am not authenticated
-    When I send a request to apply "BF2026" to the coupon API
-    Then the response is unauthorized
-    And no discount is applied
-  # ---------- AC5: Redemption record (3) ----------
-  @High @HappyPath @AC5
+  # ---------- AC4: Redemption record (3) ----------
+  @High @HappyPath @AC4
   Scenario: Redemption record is stored after a successful order
     Given I am logged in as the registered user with user_ID 5456
     And "BF2026" is applied to 1 unit of the product with product_ID 101 priced 1000.00
@@ -808,14 +837,14 @@
       | quantity discounted | 1           |
       | discount amount     | 200.00      |
       | timestamp           | current UTC |
-  @Medium @Edge @AC5
+  @Medium @Edge @AC4
   Scenario: Timestamp is stored in UTC and only 1 record is stored for quantity 2
     Given the shop time is 2026-11-28 12:00:00 (Europe/Bucharest, UTC+2)
     And "BF2026" is applied to a product with quantity 2
     When I complete the payment and the order is confirmed
     Then 1 redemption record is stored with quantity discounted = 1
     And the stored timestamp is 2026-11-28 10:00:00 UTC
-  @High @Exception @AC5
+  @High @Exception @AC4
   Scenario: Failed payment does not store a redemption and does not consume the coupon
     Given "BF2026" is applied to 1 unit of a product
     When the payment fails
@@ -866,6 +895,54 @@
     When they apply "BF2026" at the same time
     Then each request responds within the agreed time
     And every successful order stores exactly one redemption record
+  # ---------- Additional scenarios (5) ----------
+  @Medium @Alternate @AC1
+  Scenario: User removes the coupon and the original price is restored
+    Given I am logged in as a registered user with user_ID 5456
+    And my cart contains 1 unit of "Samsung Galaxy S26 Ultra 512GB" priced 1000.00
+    And I applied the coupon code "BF2026" and the order total shows 800.00
+    When I remove the coupon at Checkout
+    Then the discount line disappears
+    And the order total shows 1000.00
+    And I can apply "BF2026" again
+  @High @Exception @AC4
+  Scenario: Payment webhook retry does not create a duplicate order or redemption
+    Given I am logged in as a registered user with user_ID 5456
+    And "BF2026" is applied to 1 unit of the product with product_ID 101 priced 1000.00
+    When I pay and Stripe charges 800.00
+    And the payment confirmation webhook is delivered twice
+    Then only 1 order is created with the status "Paid"
+    And only 1 redemption record is stored with quantity discounted = 1
+    And the amount charged in Stripe equals the discounted order total of 800.00
+  @Medium @Exception @UsageLimit
+  Scenario: Cancelling the order before shipment releases the coupon
+    Given I am logged in as a registered user with user_ID 5456
+    And I completed an order with "BF2026" for the product with product_ID 101
+    And the order has not been shipped
+    When I cancel the order and the refund of 800.00 goes to the original payment method
+    Then the redemption record is flagged as cancelled
+    And I can apply "BF2026" to the product with product_ID 101 in a new order
+    # Assumption: to be confirmed with the PO (see the usage limit question on cancellation, refund, and return)
+  @High @Security @RoleBased
+  Scenario Outline: Coupon API rejects requests without a valid login token
+    Given the shop time is 2026-11-28 12:00:00
+    And a cart for user_ID 5456 contains 1 unit of a product
+    When I send a request to apply "BF2026" to the coupon API with &lt;authorization&gt;
+    Then the response is 401
+    And no discount is applied to the cart
+    Examples:
+      | authorization                        |
+      | no Authorization header              |
+      | an expired access token              |
+      | the access token of another user_ID  |
+  @Medium @Security @Negative
+  Scenario: Repeated invalid coupon attempts are rate limited
+    Given I am logged in as a registered user with 1 unit of a product at Checkout
+    When I apply 10 different invalid coupon codes within 1 minute
+    Then further attempts are blocked with a "too many attempts" message
+    And no discount is applied
+    And after the limit window I can apply "BF2026" and receive the 20% discount
+    # Assumption: the limit and the window are to be confirmed (see the invalid attempts question)
   # ---------- Regression (1) ----------
   @Medium @Regression
   Scenario: Checkout without a coupon is not affected
@@ -875,7 +952,7 @@
     And no redemption record is stored</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>**Test Case ID**: TC01
 **Title**: Apply "BF2026" to 1 unit of a smartphone
@@ -996,7 +1073,114 @@
 |----|------|----------------|
 | 1  | Add 1 unit to the cart, open Checkout and apply "BF2026". | The discount is 20.00 and the total is 80.00. |
 | 2  | Change the quantity to 3. | Only 1 unit stays discounted; the total is 280.00. |
-| 3  | Change the quantity back to 1. | The remaining unit stays discounted; the total is 80.00. |</t>
+| 3  | Change the quantity back to 1. | The remaining unit stays discounted; the total is 80.00. |
+---
+**Test Case ID**: TC08
+**Title**: Any other coupon code is rejected
+**Priority**: High
+**Objective**: Verify that invalid codes show the error message and give no discount (AC3)
+**Preconditions**:
+- The shop time is 2026-11-28 12:00 (Europe/Bucharest)
+- The user is registered and logged in
+- The cart has 1 unit of a product priced 100.00
+Test Data:
+- Codes: "BF2025", "SAVE10", "BF-2026", "BF 2026", empty, `' OR '1'='1`, `&lt;script&gt;alert(1)&lt;/script&gt;`
+Steps, Expected Results:
+| No | Step | Expected Result |
+|----|------|----------------|
+| 1  | Open Checkout and enter "BF2025", then click Apply. | The message "This coupon is not valid" is displayed and the total stays 100.00. |
+| 2  | Repeat step 1 with "SAVE10", "BF-2026" and "BF 2026". | The same message is displayed each time and no discount is applied. |
+| 3  | Click Apply with an empty field. | A validation message is displayed and no discount is applied. |
+| 4  | Enter `' OR '1'='1` and click Apply. | The message "This coupon is not valid" is displayed, with no server error. |
+| 5  | Enter `&lt;script&gt;alert(1)&lt;/script&gt;` and click Apply. | The message is displayed, no script is executed and the input is escaped. |
+| 6  | Apply "BF2026", then apply "BF2025". | The invalid message is displayed and the valid "BF2026" discount (20.00) stays applied. |
+---
+**Test Case ID**: TC09
+**Title**: Redemption record is stored after a successful order
+**Priority**: High
+**Objective**: Verify the content of the redemption record after payment (AC4)
+**Preconditions**:
+- The shop time is 2026-11-28 12:00:00 (Europe/Bucharest, UTC+2)
+- The user is registered and logged in and has not used the coupon before
+- QA can read the redemption records (DB or API)
+- Stripe test mode is used
+Test Data:
+- user_ID: 5456
+- Product: Samsung Galaxy S26 Ultra 512GB, product_ID 101, price 1000.00, qty 1
+- Stripe test card: success
+- Coupon: BF2026
+Steps, Expected Results:
+| No | Step | Expected Result |
+|----|------|----------------|
+| 1  | Add the product to the cart, open Checkout and apply "BF2026". | The discount is 200.00 and the total is 800.00. |
+| 2  | Pay with the Stripe success test card. | The payment is successful and the order confirmation page is displayed. |
+| 3  | Check the order history and the confirmation email. | The order shows the discounted total of 800.00. |
+| 4  | Read the redemption records for user_ID 5456. | Exactly 1 record exists with coupon code "BF2026", user_ID 5456, product_ID 101, quantity discounted 1, discount amount 200.00. |
+| 5  | Check the timestamp of the record. | The timestamp is stored in UTC (about 2026-11-28 10:00:00 UTC). |
+---
+**Test Case ID**: TC10
+**Title**: The same user cannot reuse the coupon for the same product, another user can
+**Priority**: High
+**Objective**: Verify the usage limit per user_ID and product
+**Preconditions**:
+- The shop time is within the promotion period
+- User A (user_ID 5456) already completed an order with "BF2026" for product_ID 101
+- User B (user_ID 7001) has not used the coupon
+Test Data:
+- Product: Samsung Galaxy S26 Ultra 512GB, product_ID 101, price 1000.00
+- Coupon: BF2026
+Steps, Expected Results:
+| No | Step | Expected Result |
+|----|------|----------------|
+| 1  | Log in as user A, add 1 unit of product_ID 101 and open Checkout. | The total is 1000.00. |
+| 2  | Apply "BF2026". | The coupon is rejected with a message (text to be confirmed) and no discount is applied. |
+| 3  | Add 1 unit of a different product (product_ID 205, charger 50.00) and apply "BF2026". | Per the agreed rule, the charger gets 10.00 off (1 discounted unit per product). |
+| 4  | Log out, log in as user B, add 1 unit of product_ID 101 and apply "BF2026". | The 20% discount of 200.00 is applied. |
+| 5  | Log in as user A again in another browser and try to apply "BF2026" for product_ID 101. | The coupon is rejected, so the limit follows the user_ID and not the browser or session. |
+---
+**Test Case ID**: TC11
+**Title**: Promotion period boundaries
+**Priority**: High
+**Objective**: Verify that the coupon is valid only between 2026-11-27 00:00:00 and 2026-11-30 23:59:59 (Europe/Bucharest)
+**Preconditions**:
+- The test environment allows setting the server date and time
+- The user is registered and logged in, and has not used the coupon
+- The cart has 1 unit of a product priced 100.00
+- The user's device clock is set to a date inside the period
+Test Data:
+- Server times: 2026-11-26 23:59:59, 2026-11-27 00:00:00, 2026-11-30 23:59:59, 2026-12-01 00:00:00
+- Coupon: BF2026
+Steps, Expected Results:
+| No | Step | Expected Result |
+|----|------|----------------|
+| 1  | Set the server time to 2026-11-26 23:59:59 and apply "BF2026". | The coupon is rejected and no discount is applied. |
+| 2  | Set the server time to 2026-11-27 00:00:00 and apply "BF2026". | The coupon is accepted and the discount is 20.00. |
+| 3  | Remove the coupon, set the server time to 2026-11-30 23:59:59 and apply "BF2026". | The coupon is accepted and the discount is 20.00. |
+| 4  | Remove the coupon, set the server time to 2026-12-01 00:00:00 and apply "BF2026". | The coupon is rejected and no discount is applied. |
+| 5  | Keep the server time at 2026-12-05 and set the device clock to 2026-11-28, then apply "BF2026". | The coupon is rejected because the server time is used. |
+---
+**Test Case ID**: TC12
+**Title**: Declined payment does not consume the coupon
+**Priority**: High
+**Objective**: Verify that a failed payment stores no redemption record, releases stock, and lets the user retry with the coupon (AC4, usage limit)
+**Preconditions**:
+- The shop time is within the promotion period
+- The user is registered and logged in and has not used the coupon before
+- Stripe test mode is used
+- The product has stock
+Test Data:
+- user_ID: 5456
+- Product: Samsung Galaxy S26 Ultra 512GB, product_ID 101, price 1000.00, qty 1
+- Stripe test cards: declined, then success
+- Coupon: BF2026
+Steps, Expected Results:
+| No | Step | Expected Result |
+|----|------|----------------|
+| 1  | Add the product to the cart, open Checkout and apply "BF2026". | The discount is 200.00 and the total is 800.00. |
+| 2  | Pay with the Stripe declined test card. | The payment fails with a clear error and no order is confirmed. |
+| 3  | Check the redemption records for user_ID 5456 and the stock of product_ID 101. | No redemption record exists and the stock is released (not deducted). |
+| 4  | Return to Checkout and check the coupon. | "BF2026" can be applied again and the discount is 200.00. |
+| 5  | Pay with the Stripe success test card. | The order is confirmed with the total 800.00, exactly 1 order is created and 1 redemption record is stored. |</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
all changes updated to the user story excel file
</commit_message>
<xml_diff>
--- a/docs/User story.xlsx
+++ b/docs/User story.xlsx
@@ -586,7 +586,26 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>- Q1: Which products are eligible: all smartphones and accessories in the catalog, or only specific categories? Are screen protectors included (they are in the description but not in AC1)? — Expected: the list of categories, and the exclusions (out-of-stock, pre-order, already discounted).
+          <t>### User Story:
+[STORY-1347] Apply Black Friday coupon code "BF2026" at checkout (full text in user-story-example.txt)
+---
+### Issues Found:
+- The product scope is listed in the description (Android and iOS smartphones, cases, screen protectors, cables, chargers), but AC1 omits screen protectors and does not say what is excluded (e.g., out-of-stock, pre-order, gift cards, already discounted items). The description also contains typos ("smarphone", "accesories", "casses", "charges").
+- The definition of "same product" is unclear: is a different color, storage size (256GB vs 512GB), or variant a different product_ID?
+- The usage limit is stated three times ("per one unit", "once per 1 unit of the same product per user_ID", "per 1 QTY of the same product for only 1 user_ID"), but it is not explicit whether the limit is per product or per campaign. The cart behavior with different products is only implied by the example.
+- AC1 and AC2 do not say which unit is discounted when units are priced differently, or how the discount is shown (line item, new total, rounding).
+- No AC for the promotion period: before 2026-11-27 00:00 or after 2026-11-30 23:59:59, there is no expected behavior or message.
+- No AC for a coupon already redeemed by the same user for the same product (second order) and no message text.
+- AC3 contradicts the validation rule: "BF2026" is case-insensitive but the AC quotes it exactly, and there is no rule for whitespace or special characters. It also does not state whether an empty code or an expired code gets the same message.
+- No AC for a failed, cancelled, or abandoned payment (is the redemption released?), or for an order cancellation, refund, or return after redemption.
+- AC4 does not say when the redemption is stored (order confirmation or payment), whether discount amount includes VAT, or how concurrent checkouts are handled.
+- The description does not say whether the coupon combines with existing promotions, sale prices, or other discounts.
+- Dependencies are not stated: the order, payment, user, and product catalog services, and the redemption storage.
+- NFRs are not addressed: security (brute-force coupon attempts, client-side tampering), performance under Black Friday load, and audit logging.
+- "User" and "registered user" are used inconsistently; the story does not say that Checkout requires a logged-in user (no guest checkout).
+---
+### Clarification &amp; Test Design Questions:
+- Q1: Which products are eligible: all smartphones and accessories in the catalog, or only specific categories? Are screen protectors included (they are in the description but not in AC1)? — Expected: the list of categories, and the exclusions (out-of-stock, pre-order, already discounted).
 - Q2: What identifies "the same product": product_ID, or product_ID plus variant (color, storage)? Is a Samsung Galaxy S26 Ultra 512GB the same product as the 256GB version? — Expected: the rule based on product_ID or SKU.
 - Q3: Is the limit "1 unit per product per user for the whole campaign" or "per order"? Can the user use the coupon again on a later order for the same product? — Expected: once per campaign, with an error message for a repeat.
 - Q4: Can the user get the discount on several different products in the same cart (e.g., a phone, a case, and a charger, each 1 unit)? Is there a cap on the number of discounted items or the total discount value? — Expected: a rule and a worked example.
@@ -602,12 +621,31 @@
 - Q14: Which UI elements show the discount (line item, new total, applied coupon label), and can the user remove the coupon? — Expected: UI/UX specification or mockup.
 - Q15: What exactly is stored in the redemption record (discount amount with or without VAT, currency, order_ID), and how can testers check it (DB, API, report)? — Expected: schema and an access method.
 - Q16: Is there a way to change the system date and to prepare test data (registered users, products, stock) in the test environment? — Expected: environment and mocking support, or a feature flag.
-- Q17: Are NFRs in scope (load on Black Friday, security of the coupon endpoint, accessibility, localization of messages, supported browsers and mobile)? — Expected: in or out of scope.</t>
+- Q17: Are NFRs in scope (load on Black Friday, security of the coupon endpoint, accessibility, localization of messages, supported browsers and mobile)? — Expected: in or out of scope.
+---
+### Suggested Test Scenarios:
+- ✅ Positive: A registered user buys 1 unit of a smartphone with "BF2026" during the period: 20% off that unit, and the redemption record is stored with correct values (AC1, AC4).
+- ✅ Positive: The same check for each accessory type: case, screen protector, cable, charger, and for both Android and iOS products.
+- ✅ Positive: "bf2026" or "Bf2026" is accepted (case-insensitive).
+- ✅ Positive: 2 units of the same product: only 1 unit discounted, the second at full price (AC2).
+- ✅ Positive: A cart with 3 different products (qty 1 each): the discount is applied per the answer to Q4.
+- ✅ Positive: Boundary times 2026-11-27 00:00:00 and 2026-11-30 23:59:59 are accepted.
+- ❌ Negative: Invalid codes ("BF2025", "SAVE10", empty, spaces, special characters, very long string, SQL/script injection) show "This coupon is not valid" (AC3).
+- ❌ Negative: 2026-11-26 23:59:59 and 2026-12-01 00:00:00 are rejected; check the UTC offset handling.
+- ❌ Negative: The same user reuses the coupon for the same product on a second order: the discount is rejected.
+- ❌ Negative: Payment fails or is cancelled: no redemption record is stored and the coupon can be reused.
+- ❌ Negative: Concurrent checkouts in two sessions: only one redemption is stored.
+- ❌ Negative: The discount is tampered with via API/DevTools (manual discount value in the request) and is rejected server-side.
+- 🔁 Regression: Checkout totals, VAT, shipping, rounding, and payment flow without a coupon.
+- 🔁 Regression: Existing promotions and discounts, the order history and invoices, and order cancellations/refunds.
+- 🔁 Regression: Login/registration flows and the cart behavior after login.
+- 🔁 Regression: Reporting/analytics and email confirmations that use the order amounts.</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>#### AC1 – Discount is applied (registered user, 1 unit)
+          <t>### Test Checklist for User Story: [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout
+#### AC1 – Discount is applied (registered user, 1 unit)
 - [ ] [AC1] Check that a registered user with 1 unit of a smartphone in the cart gets 20% off that unit after applying "BF2026" at Checkout during the promotion period
 - [ ] [AC1] Check the same for an iOS and an Android smartphone
 - [ ] [AC1] Check the same for each accessory type: case, screen protector, cable, charger
@@ -684,7 +722,38 @@
 - [ ] [Regression] Check that login and registration still work
 - [ ] [Regression] Check that order history, invoices, emails, and order cancellation/refund still show correct amounts
 - [ ] [Regression] Check that reports and analytics still work with the new redemption records
-#### Short checklist (5 items)
+### Clarification Questions
+#### Scope and product definition
+- Which products are eligible? Are screen protectors included (they are in the description but not in AC1)? Are out-of-stock, pre-order, and already discounted products excluded?
+- What identifies "the same product": product_ID only, or product_ID plus variant (color, storage)?
+#### Usage limit
+- Is the limit "1 unit per product per user for the campaign" or "per order"? Can the user use the coupon again in a later order for the same product?
+- Can the user get the discount on several different products in the same cart? Is there a cap on the total discount?
+- In AC2, which unit gets the discount when units have different prices?
+- If the order is cancelled, refunded, or the discounted unit is returned, is the coupon released for the user?
+#### Validation and messages
+- Is the code case-insensitive only, or are spaces also trimmed? Which characters are allowed?
+- Is the message "This coupon is not valid" the same for empty, unknown, and expired codes? Is there a limit on invalid attempts?
+- What message is shown when "BF2026" is used outside the promotion period?
+- What is the message when the user already used the coupon for the same product?
+#### Dates and time
+- Is 2026-11-30 23:59:59 inclusive, and which clock is used to check it? Is the check done at coupon entry, order submission, or payment?
+- What happens when the checkout starts inside the period and the payment is completed after it ends?
+#### Pricing
+- Is the 20% calculated before or after VAT? Is shipping excluded? What is the rounding rule and currency?
+- Does the coupon combine with existing sale prices, discounts, or other vouchers?
+#### Redemption record
+- When is the record stored (payment or order confirmation)? What is the amount format (with or without VAT, currency)? Is the order_ID also stored?
+- How can QA read the redemption record (DB, API, report)?
+- What happens when two checkouts of the same user complete at the same time?
+#### Non-functional and environment
+- Are performance, security, accessibility, and localization in scope for this story?
+- Can the system date be changed and test data prepared in the test environment?
+- Is a mockup or design available for the discount display at Checkout?
+#### Story quality
+- The description contains typos ("smarphone", "accesories", "casses", "charges") and the AC1 list omits screen protectors. Can the story be updated?
+- "User" and "registered user" are used inconsistently. Can the roles be defined once?
+### Test Checklist for User Story: [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout
 - [ ] [AC1/AC2] Check that a logged-in customer (user_ID 5456) with 2 units of "Samsung Galaxy S26 Ultra 512GB" at 1000.00 each gets 20% off only 1 unit after applying "BF2026" (any letter case, such as "bf2026") at Checkout. The discount is 200.00, the second unit stays at 1000.00, the total is 1800.00, and the cart, order summary and Stripe amount all match.
 - [ ] [AC3] Check that "BF2025", "SAVE10", an empty code, and injection strings (`' OR '1'='1`, `&lt;script&gt;`) show "This coupon is not valid" and apply no discount. Also check that a failed attempt does not remove an already applied valid "BF2026".
 - [ ] [Period] Check that the server time (Europe/Bucharest, UTC+2) decides validity: accepted at 2026-11-27 00:00:00 and 2026-11-30 23:59:59, rejected at 2026-11-26 23:59:59 and 2026-12-01 00:00:00, and not affected by the user's device clock.
@@ -694,7 +763,56 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Feature: Apply Black Friday coupon code "BF2026" at checkout (STORY-1347)
+          <t>## Clarity Check
+1. Which products are eligible: all smartphones and accessories, including screen protectors (listed in the description but not in AC1)? Are out-of-stock, pre-order, and already discounted products excluded?
+2. What identifies "the same product": product_ID only, or product_ID plus variant (color, storage)?
+3. Is the limit "1 unit per product per user for the whole campaign" or "per order"? Can the user use the coupon again in a later order for the same product?
+4. Can the user get the discount on several different products in the same cart? Is there a cap on the total discount?
+5. In AC2, which unit gets the discount when units have different prices?
+6. What message is shown when the code is used outside the promotion period, or when the user already redeemed the coupon for the same product?
+7. Is the code trimmed for spaces? Which characters are allowed?
+8. Is the message in AC3 the same for empty, unknown, and expired codes?
+9. If payment fails or the order is cancelled/refunded, is the coupon released and the redemption record removed?
+10. Is the 20% calculated before or after VAT? Is shipping excluded? What is the rounding rule?
+11. Does the coupon combine with other discounts or sale prices?
+12. When is the redemption record stored (payment or order confirmation)?
+*Assumptions:*
+- Eligible products are all Android and iOS smartphones and their accessories (cases, screen protectors, cables, chargers).
+- "Same product" means the same product_ID (a different variant has a different product_ID).
+- The limit is 1 discounted unit per product per user_ID for the whole campaign, so different products in the same cart each get one discounted unit.
+- The date is checked at the moment the coupon is applied and again at payment, using the server time in Europe/Bucharest. Both boundaries are inclusive.
+- The 20% is calculated on the unit price shown at checkout (with VAT); shipping is not discounted. Amounts are rounded to 2 decimals (half-up).
+- Failed or cancelled payments do not consume the coupon.
+- Codes are trimmed of leading/trailing spaces and are case-insensitive.
+- Messages outside the promotion period and for reuse are assumed: "This coupon is not valid" and "This coupon was already used for this product" (to be confirmed).
+## Detailed Analysis
+**Actor:** Registered user (customer), Product Owner (business owner of the campaign)
+**Goal:** The customer gets 20% off one unit of a product by applying coupon "BF2026" at Checkout. The Product Owner increases revenue during the Black Friday campaign.
+**Preconditions:**
+- The current shop time (Europe/Bucharest) is between 2026-11-27 00:00:00 and 2026-11-30 23:59:59.
+- The user is logged in (registered) and has at least 1 eligible product in the cart.
+- The user has not yet redeemed "BF2026" for that product.
+**Trigger:** The user enters "BF2026" on the Checkout page and clicks Apply.
+**Main Flow:**
+1. The registered user opens Checkout with 1 unit of an eligible product.
+2. The user enters "BF2026" (any letter case) and applies it.
+3. The system validates the code, the period, the user, and the usage limit.
+4. The system applies 20% off the unit and shows the discount and the new total.
+5. The user pays and the order is confirmed.
+6. The system stores a redemption record: "BF2026", user_ID, product_ID, quantity discounted = 1, discount amount, UTC timestamp.
+**Alternate Flows:**
+- Qty 2 of the same product: only 1 unit is discounted.
+- Several different products in the cart: each product gets 1 discounted unit.
+- The user changes the quantity or removes the coupon before paying.
+**Exception Flows:**
+- Invalid code: "This coupon is not valid".
+- Outside the promotion period: the coupon is rejected.
+- Coupon already used by the user for that product: the coupon is rejected.
+- Payment fails or is cancelled: no redemption record and no usage consumed.
+- The coupon service is unavailable: no discount applied.
+**Assumptions:** See the Clarity Check.
+## Test Cases
+Feature: Apply Black Friday coupon code "BF2026" at checkout (STORY-1347)
   Background:
     Given the promotion "BlackFriday2026" is configured with coupon code "BF2026" giving 20% off per 1 unit
     And the promotion period is 2026-11-27 00:00:00 to 2026-11-30 23:59:59 (Europe/Bucharest)
@@ -954,7 +1072,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>**Test Case ID**: TC01
+          <t>*Assumptions:*
+- Eligible products are all Android and iOS smartphones and their accessories (cases, screen protectors, cables, chargers).
+- "Same product" means the same product_ID; each different product gets 1 discounted unit.
+- The 20% is calculated on the unit price shown at checkout; shipping is not discounted.
+- Codes are case-insensitive and trimmed of leading/trailing spaces.
+**Test Case ID**: TC01
 **Title**: Apply "BF2026" to 1 unit of a smartphone
 **Priority**: High
 **Objective**: Verify that a registered user gets 20% off 1 unit of a smartphone (AC1)

</xml_diff>

<commit_message>
user story excel file works now
</commit_message>
<xml_diff>
--- a/docs/User story.xlsx
+++ b/docs/User story.xlsx
@@ -2,64 +2,39 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="1">
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <sz val="10"/>
-    </font>
-    <font/>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -67,55 +42,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -198,44 +138,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -262,32 +202,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -314,24 +236,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -343,162 +247,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -512,41 +420,41 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
-    <col width="80" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
     <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>User story</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>BDD test cases</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Classic test cases</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Title: [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout
 As a Product Owner, I want to start a Black Friday campaign, so that we increase our revenue on the "Smartphone-Shop" website.
@@ -584,7 +492,7 @@
 THEN the system stores a redemption record, with coupon code “BF2026”, user_ID, product_ID, quantity discounted = 1, discount amount, and a UTC timestamp.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>### User Story:
 [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout (full text in user-story-example.txt)
@@ -642,7 +550,7 @@
 - 🔁 Regression: Reporting/analytics and email confirmations that use the order amounts.</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>### Test Checklist for User Story: [STORY-1347] Apply Black Friday coupon code "BF2026" at checkout
 #### AC1 – Discount is applied (registered user, 1 unit)
@@ -761,7 +669,7 @@
 - [ ] [Security] Check that the discount cannot be changed by tampering with the request (price, discount percent, quantity, user_ID). The server must recalculate the price, reject unauthenticated or expired-token coupon requests, and rate limit repeated invalid attempts.</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>## Clarity Check
 1. Which products are eligible: all smartphones and accessories, including screen protectors (listed in the description but not in AC1)? Are out-of-stock, pre-order, and already discounted products excluded?
@@ -1070,7 +978,7 @@
     And no redemption record is stored</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>*Assumptions:*
 - Eligible products are all Android and iOS smartphones and their accessories (cases, screen protectors, cables, chargers).
@@ -1308,6 +1216,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>